<commit_message>
Week 1-Control Foundation - W1-002
</commit_message>
<xml_diff>
--- a/docs/governance/Enterprise_AI_Architecture_6_Week_Execution_Tracker_v1.3.0.xlsx
+++ b/docs/governance/Enterprise_AI_Architecture_6_Week_Execution_Tracker_v1.3.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AI\enterprise_ai_platform\docs\governance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F37201F5-CABD-46D2-A45A-83768B4D9AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1C7797C-BEE1-4A59-93F3-49425BEB992B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="903" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9955,6 +9955,18 @@
     <xf numFmtId="0" fontId="3" fillId="12" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -9962,6 +9974,24 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -9982,15 +10012,6 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -10000,20 +10021,32 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -10033,21 +10066,6 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -10056,18 +10074,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -10124,12 +10130,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -11521,48 +11521,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22.8">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="54" t="s">
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="56"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="60"/>
     </row>
     <row r="5" spans="1:10" ht="39.6">
       <c r="A5" s="21">
@@ -11574,14 +11574,14 @@
       <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="71" t="s">
+      <c r="E5" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="72"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="72"/>
-      <c r="I5" s="72"/>
-      <c r="J5" s="73"/>
+      <c r="F5" s="62"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="63"/>
     </row>
     <row r="6" spans="1:10" ht="39.6">
       <c r="A6" s="21">
@@ -11593,14 +11593,14 @@
       <c r="C6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="63" t="s">
+      <c r="E6" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="64"/>
-      <c r="G6" s="64"/>
-      <c r="H6" s="64"/>
-      <c r="I6" s="64"/>
-      <c r="J6" s="65"/>
+      <c r="F6" s="65"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="65"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="66"/>
     </row>
     <row r="7" spans="1:10" ht="52.8">
       <c r="A7" s="21">
@@ -11612,14 +11612,14 @@
       <c r="C7" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="63" t="s">
+      <c r="E7" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
-      <c r="J7" s="65"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65"/>
+      <c r="I7" s="65"/>
+      <c r="J7" s="66"/>
     </row>
     <row r="8" spans="1:10" ht="52.8">
       <c r="A8" s="21">
@@ -11631,14 +11631,14 @@
       <c r="C8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="63" t="s">
+      <c r="E8" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="64"/>
-      <c r="G8" s="64"/>
-      <c r="H8" s="64"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="65"/>
+      <c r="F8" s="65"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="65"/>
+      <c r="I8" s="65"/>
+      <c r="J8" s="66"/>
     </row>
     <row r="9" spans="1:10" ht="52.8">
       <c r="A9" s="21">
@@ -11650,14 +11650,14 @@
       <c r="C9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="64"/>
-      <c r="G9" s="64"/>
-      <c r="H9" s="64"/>
-      <c r="I9" s="64"/>
-      <c r="J9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
+      <c r="I9" s="65"/>
+      <c r="J9" s="66"/>
     </row>
     <row r="10" spans="1:10" ht="66">
       <c r="A10" s="21">
@@ -11669,14 +11669,14 @@
       <c r="C10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="63" t="s">
+      <c r="E10" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="64"/>
-      <c r="G10" s="64"/>
-      <c r="H10" s="64"/>
-      <c r="I10" s="64"/>
-      <c r="J10" s="65"/>
+      <c r="F10" s="65"/>
+      <c r="G10" s="65"/>
+      <c r="H10" s="65"/>
+      <c r="I10" s="65"/>
+      <c r="J10" s="66"/>
     </row>
     <row r="11" spans="1:10" ht="66">
       <c r="A11" s="21">
@@ -11688,14 +11688,14 @@
       <c r="C11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="66" t="s">
+      <c r="E11" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="67"/>
-      <c r="G11" s="67"/>
-      <c r="H11" s="67"/>
-      <c r="I11" s="67"/>
-      <c r="J11" s="68"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="74"/>
+      <c r="I11" s="74"/>
+      <c r="J11" s="75"/>
     </row>
     <row r="12" spans="1:10" ht="52.8">
       <c r="A12" s="21">
@@ -11721,14 +11721,14 @@
       <c r="C13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="54" t="s">
+      <c r="E13" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="55"/>
-      <c r="G13" s="55"/>
-      <c r="H13" s="55"/>
-      <c r="I13" s="55"/>
-      <c r="J13" s="56"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="59"/>
+      <c r="I13" s="59"/>
+      <c r="J13" s="60"/>
     </row>
     <row r="14" spans="1:10" ht="79.2">
       <c r="A14" s="21">
@@ -11778,38 +11778,33 @@
       </c>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="57" t="s">
+      <c r="A19" s="67" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="58"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
-      <c r="H19" s="58"/>
-      <c r="I19" s="58"/>
-      <c r="J19" s="59"/>
+      <c r="B19" s="68"/>
+      <c r="C19" s="68"/>
+      <c r="D19" s="68"/>
+      <c r="E19" s="68"/>
+      <c r="F19" s="68"/>
+      <c r="G19" s="68"/>
+      <c r="H19" s="68"/>
+      <c r="I19" s="68"/>
+      <c r="J19" s="69"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="60"/>
-      <c r="B20" s="61"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="61"/>
-      <c r="H20" s="61"/>
-      <c r="I20" s="61"/>
-      <c r="J20" s="62"/>
+      <c r="A20" s="70"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="71"/>
+      <c r="F20" s="71"/>
+      <c r="G20" s="71"/>
+      <c r="H20" s="71"/>
+      <c r="I20" s="71"/>
+      <c r="J20" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="E5:J5"/>
-    <mergeCell ref="E6:J6"/>
     <mergeCell ref="E13:J13"/>
     <mergeCell ref="A19:J20"/>
     <mergeCell ref="E7:J7"/>
@@ -11817,6 +11812,11 @@
     <mergeCell ref="E9:J9"/>
     <mergeCell ref="E10:J10"/>
     <mergeCell ref="E11:J11"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="E5:J5"/>
+    <mergeCell ref="E6:J6"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" sqref="F16" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -11843,40 +11843,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1181</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:8" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1182</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
     </row>
     <row r="4" spans="1:8" ht="46.05" customHeight="1">
-      <c r="A4" s="109" t="s">
+      <c r="A4" s="111" t="s">
         <v>1183</v>
       </c>
-      <c r="B4" s="110"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="110"/>
-      <c r="G4" s="110"/>
-      <c r="H4" s="111"/>
+      <c r="B4" s="112"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="112"/>
+      <c r="E4" s="112"/>
+      <c r="F4" s="112"/>
+      <c r="G4" s="112"/>
+      <c r="H4" s="113"/>
     </row>
     <row r="6" spans="1:8" ht="28.05" customHeight="1">
       <c r="A6" s="1" t="s">
@@ -12407,35 +12407,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.8">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="54" t="s">
         <v>1301</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="112"/>
-      <c r="J1" s="112"/>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
+      <c r="J1" s="54"/>
       <c r="K1" s="51"/>
       <c r="L1" s="51"/>
       <c r="M1" s="51"/>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="55" t="s">
         <v>1302</v>
       </c>
-      <c r="B2" s="113"/>
-      <c r="C2" s="113"/>
-      <c r="D2" s="113"/>
-      <c r="E2" s="113"/>
-      <c r="F2" s="113"/>
-      <c r="G2" s="113"/>
-      <c r="H2" s="113"/>
-      <c r="I2" s="113"/>
-      <c r="J2" s="113"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
       <c r="K2" s="52"/>
       <c r="L2" s="52"/>
       <c r="M2" s="52"/>
@@ -14067,36 +14067,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1517</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
     </row>
     <row r="2" spans="1:12" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1518</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
     </row>
     <row r="5" spans="1:12" ht="28.05" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -15249,34 +15249,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1687</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
     </row>
     <row r="2" spans="1:11" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1688</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
     </row>
     <row r="5" spans="1:11" ht="28.05" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -15948,32 +15948,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1811</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
     </row>
     <row r="2" spans="1:10" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1812</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
     </row>
     <row r="5" spans="1:10" ht="28.05" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -16768,43 +16768,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="22.8">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1892</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1893</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>1894</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="56"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="60"/>
     </row>
     <row r="5" spans="1:9" ht="26.4">
       <c r="A5" s="1" t="s">
@@ -17240,26 +17240,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1978</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
     </row>
     <row r="2" spans="1:7" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1979</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
     </row>
     <row r="5" spans="1:7" ht="28.05" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -18789,28 +18789,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>2286</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:8" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>2287</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
     </row>
     <row r="5" spans="1:8" ht="28.05" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -19651,24 +19651,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>2411</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
     </row>
     <row r="2" spans="1:6" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>2412</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
     </row>
     <row r="5" spans="1:6" ht="28.05" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -20323,144 +20323,144 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
     </row>
     <row r="2" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
+      <c r="P2" s="57"/>
     </row>
     <row r="4" spans="1:16">
-      <c r="A4" s="80" t="s">
+      <c r="A4" s="76" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="80"/>
-      <c r="D4" s="80" t="s">
+      <c r="B4" s="76"/>
+      <c r="D4" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="80"/>
-      <c r="G4" s="80" t="s">
+      <c r="E4" s="76"/>
+      <c r="G4" s="76" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="80"/>
-      <c r="J4" s="80" t="s">
+      <c r="H4" s="76"/>
+      <c r="J4" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="K4" s="80"/>
+      <c r="K4" s="76"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="81">
+      <c r="A5" s="77">
         <f>COUNTA('02 Master Plan'!$A$6:$A$120)</f>
         <v>80</v>
       </c>
-      <c r="B5" s="82"/>
-      <c r="D5" s="81">
+      <c r="B5" s="78"/>
+      <c r="D5" s="77">
         <f>COUNTIF('02 Master Plan'!$S$6:$S$120,"Done")</f>
         <v>12</v>
       </c>
-      <c r="E5" s="82"/>
-      <c r="G5" s="88">
+      <c r="E5" s="78"/>
+      <c r="G5" s="81">
         <f>IF(A5=0,0,D5/A5)</f>
         <v>0.15</v>
       </c>
-      <c r="H5" s="89"/>
-      <c r="J5" s="81">
+      <c r="H5" s="82"/>
+      <c r="J5" s="77">
         <f>COUNTIF('02 Master Plan'!$S$6:$S$120,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="K5" s="82"/>
+      <c r="K5" s="78"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="83"/>
-      <c r="B6" s="84"/>
-      <c r="D6" s="83"/>
-      <c r="E6" s="84"/>
-      <c r="G6" s="90"/>
-      <c r="H6" s="91"/>
-      <c r="J6" s="83"/>
-      <c r="K6" s="84"/>
+      <c r="A6" s="79"/>
+      <c r="B6" s="80"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="80"/>
+      <c r="G6" s="83"/>
+      <c r="H6" s="84"/>
+      <c r="J6" s="79"/>
+      <c r="K6" s="80"/>
     </row>
     <row r="7" spans="1:16">
-      <c r="A7" s="80" t="s">
+      <c r="A7" s="76" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="80"/>
-      <c r="D7" s="80" t="s">
+      <c r="B7" s="76"/>
+      <c r="D7" s="76" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="80"/>
-      <c r="G7" s="80" t="s">
+      <c r="E7" s="76"/>
+      <c r="G7" s="76" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="80"/>
-      <c r="J7" s="80" t="s">
+      <c r="H7" s="76"/>
+      <c r="J7" s="76" t="s">
         <v>52</v>
       </c>
-      <c r="K7" s="80"/>
+      <c r="K7" s="76"/>
     </row>
     <row r="8" spans="1:16">
-      <c r="A8" s="81">
+      <c r="A8" s="77">
         <f>COUNTIFS('13 Owner TODOs'!$F$6:$F$80,"&lt;&gt;Done",'13 Owner TODOs'!$A$6:$A$80,"&lt;&gt;")</f>
         <v>19</v>
       </c>
-      <c r="B8" s="82"/>
-      <c r="D8" s="81">
+      <c r="B8" s="78"/>
+      <c r="D8" s="77">
         <f>COUNTIF('11 Test Evidence'!$H$6:$H$80,"Pass")</f>
         <v>6</v>
       </c>
-      <c r="E8" s="82"/>
-      <c r="G8" s="81">
+      <c r="E8" s="78"/>
+      <c r="G8" s="77">
         <f>COUNTIF('12 Decision Log'!$C$6:$C$60,"Baseline Approved")+COUNTIF('12 Decision Log'!$C$6:$C$60,"Approved")</f>
         <v>18</v>
       </c>
-      <c r="H8" s="82"/>
-      <c r="J8" s="81">
+      <c r="H8" s="78"/>
+      <c r="J8" s="77">
         <f>COUNTIFS('11 Test Evidence'!$C$6:$C$80,"Teardown",'11 Test Evidence'!$H$6:$H$80,"Pass")</f>
         <v>1</v>
       </c>
-      <c r="K8" s="82"/>
+      <c r="K8" s="78"/>
     </row>
     <row r="9" spans="1:16">
-      <c r="A9" s="83"/>
-      <c r="B9" s="84"/>
-      <c r="D9" s="83"/>
-      <c r="E9" s="84"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="84"/>
-      <c r="J9" s="83"/>
-      <c r="K9" s="84"/>
+      <c r="A9" s="79"/>
+      <c r="B9" s="80"/>
+      <c r="D9" s="79"/>
+      <c r="E9" s="80"/>
+      <c r="G9" s="79"/>
+      <c r="H9" s="80"/>
+      <c r="J9" s="79"/>
+      <c r="K9" s="80"/>
     </row>
     <row r="12" spans="1:16" ht="28.05" customHeight="1">
       <c r="A12" s="1" t="s">
@@ -20660,89 +20660,79 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A21" s="54" t="s">
+      <c r="A21" s="58" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="55"/>
-      <c r="C21" s="55"/>
-      <c r="D21" s="55"/>
-      <c r="E21" s="55"/>
-      <c r="F21" s="55"/>
-      <c r="G21" s="55"/>
-      <c r="H21" s="56"/>
+      <c r="B21" s="59"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+      <c r="G21" s="59"/>
+      <c r="H21" s="60"/>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1">
-      <c r="A22" s="85" t="s">
+      <c r="A22" s="91" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="86"/>
-      <c r="C22" s="86"/>
-      <c r="D22" s="86"/>
-      <c r="E22" s="86"/>
-      <c r="F22" s="86"/>
-      <c r="G22" s="86"/>
-      <c r="H22" s="87"/>
+      <c r="B22" s="92"/>
+      <c r="C22" s="92"/>
+      <c r="D22" s="92"/>
+      <c r="E22" s="92"/>
+      <c r="F22" s="92"/>
+      <c r="G22" s="92"/>
+      <c r="H22" s="93"/>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1">
-      <c r="A23" s="74" t="s">
+      <c r="A23" s="85" t="s">
         <v>63</v>
       </c>
-      <c r="B23" s="75"/>
-      <c r="C23" s="75"/>
-      <c r="D23" s="75"/>
-      <c r="E23" s="75"/>
-      <c r="F23" s="75"/>
-      <c r="G23" s="75"/>
-      <c r="H23" s="76"/>
+      <c r="B23" s="86"/>
+      <c r="C23" s="86"/>
+      <c r="D23" s="86"/>
+      <c r="E23" s="86"/>
+      <c r="F23" s="86"/>
+      <c r="G23" s="86"/>
+      <c r="H23" s="87"/>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1">
-      <c r="A24" s="74" t="s">
+      <c r="A24" s="85" t="s">
         <v>64</v>
       </c>
-      <c r="B24" s="75"/>
-      <c r="C24" s="75"/>
-      <c r="D24" s="75"/>
-      <c r="E24" s="75"/>
-      <c r="F24" s="75"/>
-      <c r="G24" s="75"/>
-      <c r="H24" s="76"/>
+      <c r="B24" s="86"/>
+      <c r="C24" s="86"/>
+      <c r="D24" s="86"/>
+      <c r="E24" s="86"/>
+      <c r="F24" s="86"/>
+      <c r="G24" s="86"/>
+      <c r="H24" s="87"/>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1">
-      <c r="A25" s="74" t="s">
+      <c r="A25" s="85" t="s">
         <v>65</v>
       </c>
-      <c r="B25" s="75"/>
-      <c r="C25" s="75"/>
-      <c r="D25" s="75"/>
-      <c r="E25" s="75"/>
-      <c r="F25" s="75"/>
-      <c r="G25" s="75"/>
-      <c r="H25" s="76"/>
+      <c r="B25" s="86"/>
+      <c r="C25" s="86"/>
+      <c r="D25" s="86"/>
+      <c r="E25" s="86"/>
+      <c r="F25" s="86"/>
+      <c r="G25" s="86"/>
+      <c r="H25" s="87"/>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1">
-      <c r="A26" s="77" t="s">
+      <c r="A26" s="88" t="s">
         <v>66</v>
       </c>
-      <c r="B26" s="78"/>
-      <c r="C26" s="78"/>
-      <c r="D26" s="78"/>
-      <c r="E26" s="78"/>
-      <c r="F26" s="78"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="79"/>
+      <c r="B26" s="89"/>
+      <c r="C26" s="89"/>
+      <c r="D26" s="89"/>
+      <c r="E26" s="89"/>
+      <c r="F26" s="89"/>
+      <c r="G26" s="89"/>
+      <c r="H26" s="90"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="G5:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:K6"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A26:H26"/>
@@ -20757,6 +20747,16 @@
     <mergeCell ref="D8:E9"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G8:H9"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:K6"/>
   </mergeCells>
   <conditionalFormatting sqref="D13:D18">
     <cfRule type="dataBar" priority="1">
@@ -20855,52 +20855,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="56"/>
+      <c r="T1" s="56"/>
     </row>
     <row r="2" spans="1:21" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
-      <c r="S2" s="70"/>
-      <c r="T2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
+      <c r="P2" s="57"/>
+      <c r="Q2" s="57"/>
+      <c r="R2" s="57"/>
+      <c r="S2" s="57"/>
+      <c r="T2" s="57"/>
     </row>
     <row r="5" spans="1:21" ht="28.05" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -26085,101 +26085,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1017</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1018</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
     </row>
     <row r="4" spans="1:16" ht="28.05" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="60"/>
+      <c r="D4" s="58" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="60"/>
+      <c r="G4" s="58" t="s">
         <v>1019</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="55"/>
-      <c r="O4" s="56"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="60"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="94">
+      <c r="A5" s="96">
         <f>IF(COUNTA(O10:O40)=0,0,COUNTIF(O10:O40,"Done")/COUNTA(A10:A40))</f>
         <v>0.52173913043478259</v>
       </c>
-      <c r="B5" s="95"/>
-      <c r="D5" s="98">
+      <c r="B5" s="97"/>
+      <c r="D5" s="100">
         <f>COUNTIF(O10:O40,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="99"/>
-      <c r="G5" s="102" t="s">
+      <c r="E5" s="101"/>
+      <c r="G5" s="104" t="s">
         <v>1020</v>
       </c>
-      <c r="H5" s="103"/>
-      <c r="I5" s="103"/>
-      <c r="J5" s="103"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="103"/>
-      <c r="M5" s="103"/>
-      <c r="N5" s="103"/>
-      <c r="O5" s="104"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="106"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="101"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="107"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="99"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="108"/>
+      <c r="O6" s="109"/>
     </row>
     <row r="9" spans="1:16" ht="28.05" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -26882,21 +26882,21 @@
       </c>
     </row>
     <row r="23" spans="1:16" ht="24" customHeight="1">
-      <c r="A23" s="92"/>
-      <c r="B23" s="92"/>
-      <c r="C23" s="92"/>
-      <c r="D23" s="92"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="92"/>
-      <c r="G23" s="92"/>
-      <c r="H23" s="93"/>
-      <c r="I23" s="93"/>
-      <c r="J23" s="93"/>
-      <c r="K23" s="93"/>
-      <c r="L23" s="93"/>
-      <c r="M23" s="93"/>
-      <c r="N23" s="93"/>
-      <c r="O23" s="93"/>
+      <c r="A23" s="94"/>
+      <c r="B23" s="94"/>
+      <c r="C23" s="94"/>
+      <c r="D23" s="94"/>
+      <c r="E23" s="94"/>
+      <c r="F23" s="94"/>
+      <c r="G23" s="94"/>
+      <c r="H23" s="95"/>
+      <c r="I23" s="95"/>
+      <c r="J23" s="95"/>
+      <c r="K23" s="95"/>
+      <c r="L23" s="95"/>
+      <c r="M23" s="95"/>
+      <c r="N23" s="95"/>
+      <c r="O23" s="95"/>
     </row>
     <row r="24" spans="1:16" ht="34.049999999999997" customHeight="1">
       <c r="A24" s="30" t="s">
@@ -27179,101 +27179,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1072</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1073</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
     </row>
     <row r="4" spans="1:16" ht="28.05" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="60"/>
+      <c r="D4" s="58" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="60"/>
+      <c r="G4" s="58" t="s">
         <v>1019</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="55"/>
-      <c r="O4" s="56"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="60"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="94">
+      <c r="A5" s="96">
         <f>IF(COUNTA(O10:O40)=0,0,COUNTIF(O10:O40,"Done")/COUNTA(A10:A40))</f>
         <v>0</v>
       </c>
-      <c r="B5" s="95"/>
-      <c r="D5" s="98">
+      <c r="B5" s="97"/>
+      <c r="D5" s="100">
         <f>COUNTIF(O10:O40,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="99"/>
-      <c r="G5" s="102" t="s">
+      <c r="E5" s="101"/>
+      <c r="G5" s="104" t="s">
         <v>1074</v>
       </c>
-      <c r="H5" s="103"/>
-      <c r="I5" s="103"/>
-      <c r="J5" s="103"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="103"/>
-      <c r="M5" s="103"/>
-      <c r="N5" s="103"/>
-      <c r="O5" s="104"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="106"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="101"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="107"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="99"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="108"/>
+      <c r="O6" s="109"/>
     </row>
     <row r="9" spans="1:16" ht="28.05" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -27976,21 +27976,21 @@
       </c>
     </row>
     <row r="23" spans="1:16" ht="24" customHeight="1">
-      <c r="A23" s="92"/>
-      <c r="B23" s="92"/>
-      <c r="C23" s="92"/>
-      <c r="D23" s="92"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="92"/>
-      <c r="G23" s="92"/>
-      <c r="H23" s="93"/>
-      <c r="I23" s="93"/>
-      <c r="J23" s="93"/>
-      <c r="K23" s="93"/>
-      <c r="L23" s="93"/>
-      <c r="M23" s="93"/>
-      <c r="N23" s="93"/>
-      <c r="O23" s="93"/>
+      <c r="A23" s="94"/>
+      <c r="B23" s="94"/>
+      <c r="C23" s="94"/>
+      <c r="D23" s="94"/>
+      <c r="E23" s="94"/>
+      <c r="F23" s="94"/>
+      <c r="G23" s="94"/>
+      <c r="H23" s="95"/>
+      <c r="I23" s="95"/>
+      <c r="J23" s="95"/>
+      <c r="K23" s="95"/>
+      <c r="L23" s="95"/>
+      <c r="M23" s="95"/>
+      <c r="N23" s="95"/>
+      <c r="O23" s="95"/>
     </row>
     <row r="24" spans="1:16" ht="34.049999999999997" customHeight="1">
       <c r="A24" s="30" t="s">
@@ -28250,101 +28250,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1097</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1098</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
     </row>
     <row r="4" spans="1:16" ht="28.05" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="60"/>
+      <c r="D4" s="58" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="60"/>
+      <c r="G4" s="58" t="s">
         <v>1019</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="55"/>
-      <c r="O4" s="56"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="60"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="94">
+      <c r="A5" s="96">
         <f>IF(COUNTA(O10:O40)=0,0,COUNTIF(O10:O40,"Done")/COUNTA(A10:A40))</f>
         <v>0</v>
       </c>
-      <c r="B5" s="95"/>
-      <c r="D5" s="98">
+      <c r="B5" s="97"/>
+      <c r="D5" s="100">
         <f>COUNTIF(O10:O40,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="99"/>
-      <c r="G5" s="102" t="s">
+      <c r="E5" s="101"/>
+      <c r="G5" s="104" t="s">
         <v>1099</v>
       </c>
-      <c r="H5" s="103"/>
-      <c r="I5" s="103"/>
-      <c r="J5" s="103"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="103"/>
-      <c r="M5" s="103"/>
-      <c r="N5" s="103"/>
-      <c r="O5" s="104"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="106"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="101"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="107"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="99"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="108"/>
+      <c r="O6" s="109"/>
     </row>
     <row r="9" spans="1:16" ht="28.05" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -29047,21 +29047,21 @@
       </c>
     </row>
     <row r="23" spans="1:16" ht="24" customHeight="1">
-      <c r="A23" s="92"/>
-      <c r="B23" s="92"/>
-      <c r="C23" s="92"/>
-      <c r="D23" s="92"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="92"/>
-      <c r="G23" s="92"/>
-      <c r="H23" s="93"/>
-      <c r="I23" s="93"/>
-      <c r="J23" s="93"/>
-      <c r="K23" s="93"/>
-      <c r="L23" s="93"/>
-      <c r="M23" s="93"/>
-      <c r="N23" s="93"/>
-      <c r="O23" s="93"/>
+      <c r="A23" s="94"/>
+      <c r="B23" s="94"/>
+      <c r="C23" s="94"/>
+      <c r="D23" s="94"/>
+      <c r="E23" s="94"/>
+      <c r="F23" s="94"/>
+      <c r="G23" s="94"/>
+      <c r="H23" s="95"/>
+      <c r="I23" s="95"/>
+      <c r="J23" s="95"/>
+      <c r="K23" s="95"/>
+      <c r="L23" s="95"/>
+      <c r="M23" s="95"/>
+      <c r="N23" s="95"/>
+      <c r="O23" s="95"/>
     </row>
     <row r="24" spans="1:16" ht="34.049999999999997" customHeight="1">
       <c r="A24" s="30" t="s">
@@ -29298,101 +29298,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1118</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1119</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
     </row>
     <row r="4" spans="1:16" ht="28.05" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="60"/>
+      <c r="D4" s="58" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="60"/>
+      <c r="G4" s="58" t="s">
         <v>1019</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="55"/>
-      <c r="O4" s="56"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="60"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="94">
+      <c r="A5" s="96">
         <f>IF(COUNTA(O10:O40)=0,0,COUNTIF(O10:O40,"Done")/COUNTA(A10:A40))</f>
         <v>0</v>
       </c>
-      <c r="B5" s="95"/>
-      <c r="D5" s="98">
+      <c r="B5" s="97"/>
+      <c r="D5" s="100">
         <f>COUNTIF(O10:O40,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="99"/>
-      <c r="G5" s="102" t="s">
+      <c r="E5" s="101"/>
+      <c r="G5" s="104" t="s">
         <v>1120</v>
       </c>
-      <c r="H5" s="103"/>
-      <c r="I5" s="103"/>
-      <c r="J5" s="103"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="103"/>
-      <c r="M5" s="103"/>
-      <c r="N5" s="103"/>
-      <c r="O5" s="104"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="106"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="101"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="107"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="99"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="108"/>
+      <c r="O6" s="109"/>
     </row>
     <row r="9" spans="1:16" ht="28.05" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -30095,21 +30095,21 @@
       </c>
     </row>
     <row r="23" spans="1:16" ht="24" customHeight="1">
-      <c r="A23" s="92"/>
-      <c r="B23" s="92"/>
-      <c r="C23" s="92"/>
-      <c r="D23" s="92"/>
-      <c r="E23" s="92"/>
-      <c r="F23" s="92"/>
-      <c r="G23" s="92"/>
-      <c r="H23" s="93"/>
-      <c r="I23" s="93"/>
-      <c r="J23" s="93"/>
-      <c r="K23" s="93"/>
-      <c r="L23" s="93"/>
-      <c r="M23" s="93"/>
-      <c r="N23" s="93"/>
-      <c r="O23" s="93"/>
+      <c r="A23" s="94"/>
+      <c r="B23" s="94"/>
+      <c r="C23" s="94"/>
+      <c r="D23" s="94"/>
+      <c r="E23" s="94"/>
+      <c r="F23" s="94"/>
+      <c r="G23" s="94"/>
+      <c r="H23" s="95"/>
+      <c r="I23" s="95"/>
+      <c r="J23" s="95"/>
+      <c r="K23" s="95"/>
+      <c r="L23" s="95"/>
+      <c r="M23" s="95"/>
+      <c r="N23" s="95"/>
+      <c r="O23" s="95"/>
     </row>
     <row r="24" spans="1:16" ht="34.049999999999997" customHeight="1">
       <c r="A24" s="30" t="s">
@@ -30346,101 +30346,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1139</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1140</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
     </row>
     <row r="4" spans="1:16" ht="28.05" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="60"/>
+      <c r="D4" s="58" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="60"/>
+      <c r="G4" s="58" t="s">
         <v>1019</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="55"/>
-      <c r="O4" s="56"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="60"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="94">
+      <c r="A5" s="96">
         <f>IF(COUNTA(O10:O40)=0,0,COUNTIF(O10:O40,"Done")/COUNTA(A10:A40))</f>
         <v>0</v>
       </c>
-      <c r="B5" s="95"/>
-      <c r="D5" s="98">
+      <c r="B5" s="97"/>
+      <c r="D5" s="100">
         <f>COUNTIF(O10:O40,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="99"/>
-      <c r="G5" s="102" t="s">
+      <c r="E5" s="101"/>
+      <c r="G5" s="104" t="s">
         <v>1141</v>
       </c>
-      <c r="H5" s="103"/>
-      <c r="I5" s="103"/>
-      <c r="J5" s="103"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="103"/>
-      <c r="M5" s="103"/>
-      <c r="N5" s="103"/>
-      <c r="O5" s="104"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="106"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="101"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="107"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="99"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="108"/>
+      <c r="O6" s="109"/>
     </row>
     <row r="9" spans="1:16" ht="28.05" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -31193,21 +31193,21 @@
       </c>
     </row>
     <row r="24" spans="1:16" ht="34.049999999999997" customHeight="1">
-      <c r="A24" s="108"/>
-      <c r="B24" s="108"/>
-      <c r="C24" s="108"/>
-      <c r="D24" s="108"/>
-      <c r="E24" s="108"/>
-      <c r="F24" s="108"/>
-      <c r="G24" s="108"/>
-      <c r="H24" s="93"/>
-      <c r="I24" s="93"/>
-      <c r="J24" s="93"/>
-      <c r="K24" s="93"/>
-      <c r="L24" s="93"/>
-      <c r="M24" s="93"/>
-      <c r="N24" s="93"/>
-      <c r="O24" s="93"/>
+      <c r="A24" s="110"/>
+      <c r="B24" s="110"/>
+      <c r="C24" s="110"/>
+      <c r="D24" s="110"/>
+      <c r="E24" s="110"/>
+      <c r="F24" s="110"/>
+      <c r="G24" s="110"/>
+      <c r="H24" s="95"/>
+      <c r="I24" s="95"/>
+      <c r="J24" s="95"/>
+      <c r="K24" s="95"/>
+      <c r="L24" s="95"/>
+      <c r="M24" s="95"/>
+      <c r="N24" s="95"/>
+      <c r="O24" s="95"/>
     </row>
     <row r="25" spans="1:16" ht="48" customHeight="1">
       <c r="A25" s="32" t="s">
@@ -31467,101 +31467,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="56" t="s">
         <v>1164</v>
       </c>
-      <c r="B1" s="69"/>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:16" ht="31.95" customHeight="1">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="57" t="s">
         <v>1165</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
     </row>
     <row r="4" spans="1:16" ht="28.05" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="60"/>
+      <c r="D4" s="58" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="60"/>
+      <c r="G4" s="58" t="s">
         <v>1019</v>
       </c>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55"/>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="55"/>
-      <c r="O4" s="56"/>
+      <c r="H4" s="59"/>
+      <c r="I4" s="59"/>
+      <c r="J4" s="59"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="59"/>
+      <c r="N4" s="59"/>
+      <c r="O4" s="60"/>
     </row>
     <row r="5" spans="1:16">
-      <c r="A5" s="94">
+      <c r="A5" s="96">
         <f>IF(COUNTA(O10:O40)=0,0,COUNTIF(O10:O40,"Done")/COUNTA(A10:A40))</f>
         <v>0</v>
       </c>
-      <c r="B5" s="95"/>
-      <c r="D5" s="98">
+      <c r="B5" s="97"/>
+      <c r="D5" s="100">
         <f>COUNTIF(O10:O40,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="99"/>
-      <c r="G5" s="102" t="s">
+      <c r="E5" s="101"/>
+      <c r="G5" s="104" t="s">
         <v>1166</v>
       </c>
-      <c r="H5" s="103"/>
-      <c r="I5" s="103"/>
-      <c r="J5" s="103"/>
-      <c r="K5" s="103"/>
-      <c r="L5" s="103"/>
-      <c r="M5" s="103"/>
-      <c r="N5" s="103"/>
-      <c r="O5" s="104"/>
+      <c r="H5" s="105"/>
+      <c r="I5" s="105"/>
+      <c r="J5" s="105"/>
+      <c r="K5" s="105"/>
+      <c r="L5" s="105"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="105"/>
+      <c r="O5" s="106"/>
     </row>
     <row r="6" spans="1:16">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
-      <c r="D6" s="100"/>
-      <c r="E6" s="101"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="106"/>
-      <c r="I6" s="106"/>
-      <c r="J6" s="106"/>
-      <c r="K6" s="106"/>
-      <c r="L6" s="106"/>
-      <c r="M6" s="106"/>
-      <c r="N6" s="106"/>
-      <c r="O6" s="107"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="99"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="103"/>
+      <c r="G6" s="107"/>
+      <c r="H6" s="108"/>
+      <c r="I6" s="108"/>
+      <c r="J6" s="108"/>
+      <c r="K6" s="108"/>
+      <c r="L6" s="108"/>
+      <c r="M6" s="108"/>
+      <c r="N6" s="108"/>
+      <c r="O6" s="109"/>
     </row>
     <row r="9" spans="1:16" ht="28.05" customHeight="1">
       <c r="A9" s="1" t="s">
@@ -32314,21 +32314,21 @@
       </c>
     </row>
     <row r="24" spans="1:16" ht="34.049999999999997" customHeight="1">
-      <c r="A24" s="108"/>
-      <c r="B24" s="108"/>
-      <c r="C24" s="108"/>
-      <c r="D24" s="108"/>
-      <c r="E24" s="108"/>
-      <c r="F24" s="108"/>
-      <c r="G24" s="108"/>
-      <c r="H24" s="93"/>
-      <c r="I24" s="93"/>
-      <c r="J24" s="93"/>
-      <c r="K24" s="93"/>
-      <c r="L24" s="93"/>
-      <c r="M24" s="93"/>
-      <c r="N24" s="93"/>
-      <c r="O24" s="93"/>
+      <c r="A24" s="110"/>
+      <c r="B24" s="110"/>
+      <c r="C24" s="110"/>
+      <c r="D24" s="110"/>
+      <c r="E24" s="110"/>
+      <c r="F24" s="110"/>
+      <c r="G24" s="110"/>
+      <c r="H24" s="95"/>
+      <c r="I24" s="95"/>
+      <c r="J24" s="95"/>
+      <c r="K24" s="95"/>
+      <c r="L24" s="95"/>
+      <c r="M24" s="95"/>
+      <c r="N24" s="95"/>
+      <c r="O24" s="95"/>
     </row>
     <row r="25" spans="1:16" ht="48" customHeight="1">
       <c r="A25" s="32" t="s">

</xml_diff>